<commit_message>
Finished coding changes to treatment. Now testing code.
</commit_message>
<xml_diff>
--- a/resources/Intervention_parameters_local.xlsx
+++ b/resources/Intervention_parameters_local.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://imperiallondon-my.sharepoint.com/personal/mpickles_ic_ac_uk/Documents/Dropbox_copy/Hepatitis B/Modelling/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="70" documentId="13_ncr:1_{27784630-3534-4B11-A251-D9C00B8973FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FC79DF7A-C723-4BA4-8D80-7299E3A5DCCD}"/>
+  <xr:revisionPtr revIDLastSave="245" documentId="13_ncr:1_{27784630-3534-4B11-A251-D9C00B8973FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1D9D8FF1-47F5-44FF-A2D1-4D75A91D6986}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{32AE504A-42D4-4D2F-BBAF-CD32E5E95CB5}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="2" xr2:uid="{32AE504A-42D4-4D2F-BBAF-CD32E5E95CB5}"/>
   </bookViews>
   <sheets>
     <sheet name="Scenario_descriptions" sheetId="4" r:id="rId1"/>
@@ -19,6 +19,9 @@
     <sheet name="WHO_region_parameters" sheetId="2" r:id="rId4"/>
     <sheet name="Notes" sheetId="5" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName name="Dx_infacilitytesting_acceptability">GlobalParams!$B$18</definedName>
+  </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -43,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="414">
   <si>
     <t>Scenario index</t>
   </si>
@@ -247,12 +250,6 @@
     <t>ContImp + Integrated services</t>
   </si>
   <si>
-    <t>TBD - HIV (or triple elimination)?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bulstra PLoS Med 2021, Integrating HIV services and other health services: A systematic review and meta- Analysis. </t>
-  </si>
-  <si>
     <t>CompInt + PoC Tx eligibility</t>
   </si>
   <si>
@@ -1009,13 +1006,7 @@
     <t>BD_in_facility_acceptance_contimp</t>
   </si>
   <si>
-    <t>Median of BD/in-facility births across countries with BD</t>
-  </si>
-  <si>
     <t>BD_oof_coverage</t>
-  </si>
-  <si>
-    <t>Assumption: effective coverage for OOF facility births can reach 60% through given mechanism used (e.g. MAP, CHWs)</t>
   </si>
   <si>
     <t>HepB3_WHO_target_coverage</t>
@@ -1192,12 +1183,201 @@
   <si>
     <t>Nicaragua</t>
   </si>
+  <si>
+    <t>Decentralisation_prop_rural</t>
+  </si>
+  <si>
+    <t>Integrated service delivery models - look at Stockdale review L GastroHep 2025, see which of the reviewed articles seems closest.</t>
+  </si>
+  <si>
+    <t>PoC eligibility - B-simple. Check if Shevanthi can get the B-simple study protocol with power calculations for effect size</t>
+  </si>
+  <si>
+    <t>Across countries I can look at whether HIV or non-communicable diseases has a bigger coverage, and use that?</t>
+  </si>
+  <si>
+    <t>Opt-out testing: https://pubmed.ncbi.nlm.nih.gov/35702813/ is UK based for EDs (+similar) finding uptake 16-91%.</t>
+  </si>
+  <si>
+    <t>Note - 69 countries have WHS, but 13 high-income (European) don't have section 7. In addition Turkiye should have that data but it is not in the dataset (and the report contains empty tables and blank pages!)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Data/WHS_WHO/WHS_analysis.R (and Data/WHS_WHO/WHS_preliminary_analysis.R). The former generates </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>WHS_utilization.csv</t>
+    </r>
+  </si>
+  <si>
+    <t>Prop_access_healthservices</t>
+  </si>
+  <si>
+    <t>Dx_infacilitytesting_acceptability</t>
+  </si>
+  <si>
+    <t>Two reviews for high-income settings found a wide range of acceptability in EDs (Simmons HIV Med 2022 - 16-91%; Metcalfe HIV Med 2026 20-75%) so take rough mid-point</t>
+  </si>
+  <si>
+    <t>Dx_coverage_with_infacilitytesting</t>
+  </si>
+  <si>
+    <t>Bulstra PLoS Med 2021, Integrating HIV services and other health services: A systematic review and meta- Analysis. 
+Triple elimination: https://www.clintonhealthaccess.org/wp-content/uploads/2026/03/CHAI-Integrated-Screening-Market-Memo-March-2026.pdf
+Look at NCD and HIV service coverage indicators</t>
+  </si>
+  <si>
+    <t>TBD - HIV (or triple elimination)? Look at NCD or HIV indicators</t>
+  </si>
+  <si>
+    <t>Proportion of in-facility births where the mother will accept BD</t>
+  </si>
+  <si>
+    <t>Proportion of OOFs which can get BD through some mechanism (e.g. MAP, CHWs)</t>
+  </si>
+  <si>
+    <t>Value is median of BD/in-facility births across countries with BD</t>
+  </si>
+  <si>
+    <t>Find the script/line that does this.</t>
+  </si>
+  <si>
+    <t>The target for HepB3 coverage under scenarios increasing Hep B3 - we take this to be the WHO target (as HepB3 coverage is already high)</t>
+  </si>
+  <si>
+    <t>The start of the HepB3 intervention.</t>
+  </si>
+  <si>
+    <t>The time at which the HepB3 intervention reaches the target value.</t>
+  </si>
+  <si>
+    <t>The sensitivity of the point-of-care test used for PAP eligibility (i.e. to determine high VL)</t>
+  </si>
+  <si>
+    <t>The sensitivity of the PoC PAP test</t>
+  </si>
+  <si>
+    <t>Start of birth cohort testing (when used)</t>
+  </si>
+  <si>
+    <t>End of birth cohort testing (when used)</t>
+  </si>
+  <si>
+    <t>Start of community screening testing (when used)</t>
+  </si>
+  <si>
+    <t>End of community screening testing (when used)</t>
+  </si>
+  <si>
+    <t>Coverage of community screening (when used)</t>
+  </si>
+  <si>
+    <t>Probably should be longer than birth cohort testing</t>
+  </si>
+  <si>
+    <t>Extras</t>
+  </si>
+  <si>
+    <t>RRprogress_effective_TDFtreatment_nonCC</t>
+  </si>
+  <si>
+    <t>RRprogress_effective_TDFtreatment_CC</t>
+  </si>
+  <si>
+    <t>Relative rate of progression from one stage to the next when on effective tenofovir treatment (excluding developing CC/death)</t>
+  </si>
+  <si>
+    <t>Relative rate of progression from stage to CC or death when on effective tenofovir treatment</t>
+  </si>
+  <si>
+    <t>Relative rate of progression from one stage to the next when on tenofovir treatment but not adherent (excluding developing CC/death)</t>
+  </si>
+  <si>
+    <t>Relative rate of progression from stage to CC or death when on tenofovir treatment but not adherent</t>
+  </si>
+  <si>
+    <t>RRprogress_nonadherent_TDFtreatment_nonCC</t>
+  </si>
+  <si>
+    <t>RRprogress_nonadherent_TDFtreatment_CC</t>
+  </si>
+  <si>
+    <t>RRprogress_effective_LAtreatment_CC</t>
+  </si>
+  <si>
+    <t>RRprogress_nonadherent_LAtreatment_nonCC</t>
+  </si>
+  <si>
+    <t>RRprogress_nonadherent_LAtreatment_CC</t>
+  </si>
+  <si>
+    <t>RRprogress_effective_LAtreatment_nonCC</t>
+  </si>
+  <si>
+    <t>Relative rate of progression from one stage to the next when on effective long-acting treatment (excluding developing CC/death)</t>
+  </si>
+  <si>
+    <t>Relative rate of progression from stage to CC or death when on effective long-acting treatment</t>
+  </si>
+  <si>
+    <t>Relative rate of progression from one stage to the next when on long-acting treatment but not adherent (excluding developing CC/death)</t>
+  </si>
+  <si>
+    <t>Relative rate of progression from stage to CC or death when on long-acting treatment but not adherent</t>
+  </si>
+  <si>
+    <t>RRtrans_effective_LAtreatment</t>
+  </si>
+  <si>
+    <t>RRtrans_nonadherent_LAtreatment</t>
+  </si>
+  <si>
+    <t>RRtrans_effective_TDFtreatment</t>
+  </si>
+  <si>
+    <t>RRtrans_nonadherent_TDFtreatment</t>
+  </si>
+  <si>
+    <t>Relative risk of transmission from someone on effective LA treatment (compared to not on treatment)</t>
+  </si>
+  <si>
+    <t>Relative risk of transmission from someone on LA treatment but not adherent (compared to not on treatment)</t>
+  </si>
+  <si>
+    <t>Relative risk of transmission from someone on (current) TDF treatment but not adherent (compared to not on treatment)</t>
+  </si>
+  <si>
+    <t>Relative risk of transmission from someone on effective (current) TDF treatment (compared to not on treatment)</t>
+  </si>
+  <si>
+    <t>Coverage of testing (accepts test and collects results) among those in the birth cohort when birth cohort testing used</t>
+  </si>
+  <si>
+    <t>prop_adhere_current</t>
+  </si>
+  <si>
+    <t>Proportion of people who, when diagnosed and eligible, start effective treatment</t>
+  </si>
+  <si>
+    <t>prop_nonadhere_current</t>
+  </si>
+  <si>
+    <t>Proportion of people who, when diagnosed and eligible, start non-adherent treatment - the proportion who go out of care is then 1-(prop_adhere_current+prop_nonadhere_current)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1252,8 +1432,20 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FF000000"/>
+      <name val="Lucida Console"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FFBCBCBC"/>
+      <name val="Lucida Console"/>
+      <family val="3"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1272,6 +1464,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1286,7 +1484,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1313,6 +1511,15 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1857,7 +2064,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>43</v>
@@ -1891,16 +2098,22 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>50</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>334</v>
+        <v>330</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1908,16 +2121,16 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="E15" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1925,13 +2138,13 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>51</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1945,10 +2158,10 @@
         <v>53</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="G17" t="s">
-        <v>55</v>
+        <v>368</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>367</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1956,16 +2169,16 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D18" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="E18" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1973,13 +2186,13 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
+        <v>55</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D19" t="s">
         <v>57</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D19" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1987,16 +2200,16 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D20" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2004,16 +2217,16 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
+        <v>60</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D21" t="s">
         <v>62</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="E21" s="2" t="s">
         <v>63</v>
-      </c>
-      <c r="D21" t="s">
-        <v>64</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -2021,16 +2234,16 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
+        <v>342</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="D22" t="s">
         <v>346</v>
       </c>
-      <c r="C22" s="2" t="s">
-        <v>348</v>
-      </c>
-      <c r="D22" t="s">
-        <v>350</v>
-      </c>
       <c r="E22" s="2" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
@@ -2038,16 +2251,16 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
+        <v>343</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="D23" t="s">
         <v>347</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>349</v>
-      </c>
-      <c r="D23" t="s">
-        <v>351</v>
-      </c>
       <c r="E23" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
     </row>
   </sheetData>
@@ -2058,7 +2271,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55F8FC61-4B68-4337-A066-5076E487245E}">
-  <dimension ref="A1:M111"/>
+  <dimension ref="A1:O111"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4.81640625" bestFit="1" customWidth="1"/>
@@ -2072,58 +2285,66 @@
     <col min="9" max="9" width="28.54296875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16.54296875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="26" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="24.36328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="30.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>77</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="B2" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="C2" t="s">
         <v>79</v>
-      </c>
-      <c r="B2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C2" t="s">
-        <v>81</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -2157,16 +2378,23 @@
       <c r="M2">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N2">
+        <v>0.16919000000000001</v>
+      </c>
+      <c r="O2">
+        <f>VLOOKUP(C2,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.34718290865108348</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C3" t="s">
         <v>82</v>
-      </c>
-      <c r="B3" t="s">
-        <v>83</v>
-      </c>
-      <c r="C3" t="s">
-        <v>84</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -2200,16 +2428,23 @@
       <c r="M3">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N3">
+        <v>0.24034</v>
+      </c>
+      <c r="O3">
+        <f>VLOOKUP(C3,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B4" t="s">
+        <v>84</v>
+      </c>
+      <c r="C4" t="s">
         <v>85</v>
-      </c>
-      <c r="B4" t="s">
-        <v>86</v>
-      </c>
-      <c r="C4" t="s">
-        <v>87</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -2243,16 +2478,23 @@
       <c r="M4">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N4">
+        <v>0.30967</v>
+      </c>
+      <c r="O4">
+        <f>VLOOKUP(C4,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.42042078352794848</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B5" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -2286,16 +2528,23 @@
       <c r="M5">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N5">
+        <v>0.22591999999999998</v>
+      </c>
+      <c r="O5">
+        <f>VLOOKUP(C5,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.42042078352794848</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B6" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -2329,16 +2578,23 @@
       <c r="M6">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N6">
+        <v>0.20919000000000001</v>
+      </c>
+      <c r="O6">
+        <f>VLOOKUP(C6,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.42042078352794848</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B7" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C7" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D7">
         <v>0</v>
@@ -2372,16 +2628,23 @@
       <c r="M7">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N7">
+        <v>0.10798999999999999</v>
+      </c>
+      <c r="O7">
+        <f>VLOOKUP(C7,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B8" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C8" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D8">
         <v>0</v>
@@ -2415,16 +2678,23 @@
       <c r="M8">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N8">
+        <v>0.2586</v>
+      </c>
+      <c r="O8">
+        <f>VLOOKUP(C8,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B9" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C9" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D9">
         <v>0</v>
@@ -2458,16 +2728,23 @@
       <c r="M9">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N9">
+        <v>0.48347999999999997</v>
+      </c>
+      <c r="O9">
+        <f>VLOOKUP(C9,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
+        <v>96</v>
+      </c>
+      <c r="B10" t="s">
+        <v>97</v>
+      </c>
+      <c r="C10" t="s">
         <v>98</v>
-      </c>
-      <c r="B10" t="s">
-        <v>99</v>
-      </c>
-      <c r="C10" t="s">
-        <v>100</v>
       </c>
       <c r="D10">
         <v>0</v>
@@ -2501,16 +2778,23 @@
       <c r="M10">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N10">
+        <v>1.9879999999999998E-2</v>
+      </c>
+      <c r="O10">
+        <f>VLOOKUP(C10,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.35465693889566102</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B11" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C11" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D11">
         <v>0</v>
@@ -2544,16 +2828,23 @@
       <c r="M11">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N11">
+        <v>0.48316000000000003</v>
+      </c>
+      <c r="O11">
+        <f>VLOOKUP(C11,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.42042078352794848</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B12" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D12">
         <v>0</v>
@@ -2587,16 +2878,23 @@
       <c r="M12">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N12">
+        <v>0.24876000000000001</v>
+      </c>
+      <c r="O12">
+        <f>VLOOKUP(C12,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.42042078352794848</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
+        <v>103</v>
+      </c>
+      <c r="B13" t="s">
+        <v>104</v>
+      </c>
+      <c r="C13" t="s">
         <v>105</v>
-      </c>
-      <c r="B13" t="s">
-        <v>106</v>
-      </c>
-      <c r="C13" t="s">
-        <v>107</v>
       </c>
       <c r="D13">
         <v>0</v>
@@ -2630,16 +2928,23 @@
       <c r="M13">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N13">
+        <v>0.41054000000000002</v>
+      </c>
+      <c r="O13">
+        <f>VLOOKUP(C13,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.426962734427077</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B14" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C14" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D14">
         <v>0</v>
@@ -2673,16 +2978,23 @@
       <c r="M14">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N14">
+        <v>0.27587</v>
+      </c>
+      <c r="O14">
+        <f>VLOOKUP(C14,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.426962734427077</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B15" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C15" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D15">
         <v>0</v>
@@ -2716,16 +3028,23 @@
       <c r="M15">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N15">
+        <v>0.67525999999999997</v>
+      </c>
+      <c r="O15">
+        <f>VLOOKUP(C15,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.35465693889566102</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B16" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C16" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D16">
         <v>0</v>
@@ -2759,16 +3078,23 @@
       <c r="M16">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N16">
+        <v>0.44543999999999995</v>
+      </c>
+      <c r="O16">
+        <f>VLOOKUP(C16,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
+        <v>112</v>
+      </c>
+      <c r="B17" t="s">
+        <v>113</v>
+      </c>
+      <c r="C17" t="s">
         <v>114</v>
-      </c>
-      <c r="B17" t="s">
-        <v>115</v>
-      </c>
-      <c r="C17" t="s">
-        <v>116</v>
       </c>
       <c r="D17">
         <v>0</v>
@@ -2802,16 +3128,23 @@
       <c r="M17">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N17">
+        <v>0.1628</v>
+      </c>
+      <c r="O17">
+        <f>VLOOKUP(C17,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.28018755337085549</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B18" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C18" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D18">
         <v>0</v>
@@ -2845,16 +3178,23 @@
       <c r="M18">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N18">
+        <v>0.31069999999999998</v>
+      </c>
+      <c r="O18">
+        <f>VLOOKUP(C18,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B19" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C19" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D19">
         <v>0</v>
@@ -2888,16 +3228,23 @@
       <c r="M19">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N19">
+        <v>0.24193000000000001</v>
+      </c>
+      <c r="O19">
+        <f>VLOOKUP(C19,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B20" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C20" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D20">
         <v>0</v>
@@ -2931,16 +3278,23 @@
       <c r="M20">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N20">
+        <v>0.26267000000000001</v>
+      </c>
+      <c r="O20">
+        <f>VLOOKUP(C20,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B21" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C21" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D21">
         <v>0</v>
@@ -2974,16 +3328,23 @@
       <c r="M21">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N21">
+        <v>8.1110000000000002E-2</v>
+      </c>
+      <c r="O21">
+        <f>VLOOKUP(C21,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B22" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C22" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D22">
         <v>0</v>
@@ -3017,16 +3378,23 @@
       <c r="M22">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N22">
+        <v>0.17756</v>
+      </c>
+      <c r="O22">
+        <f>VLOOKUP(C22,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.426962734427077</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B23" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C23" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D23">
         <v>0</v>
@@ -3060,16 +3428,23 @@
       <c r="M23">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N23">
+        <v>0.12445000000000001</v>
+      </c>
+      <c r="O23">
+        <f>VLOOKUP(C23,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B24" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C24" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D24">
         <v>0</v>
@@ -3103,16 +3478,23 @@
       <c r="M24">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N24">
+        <v>0.27032</v>
+      </c>
+      <c r="O24">
+        <f>VLOOKUP(C24,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B25" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C25" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D25">
         <v>0</v>
@@ -3146,16 +3528,23 @@
       <c r="M25">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N25">
+        <v>0.17492999999999997</v>
+      </c>
+      <c r="O25">
+        <f>VLOOKUP(C25,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.426962734427077</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B26" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C26" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D26">
         <v>0</v>
@@ -3189,16 +3578,23 @@
       <c r="M26">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N26">
+        <v>0.10621999999999999</v>
+      </c>
+      <c r="O26">
+        <f>VLOOKUP(C26,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.34718290865108348</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B27" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C27" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D27">
         <v>0</v>
@@ -3232,16 +3628,23 @@
       <c r="M27">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N27">
+        <v>0.19</v>
+      </c>
+      <c r="O27">
+        <f>VLOOKUP(C27,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B28" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C28" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D28">
         <v>0</v>
@@ -3275,16 +3678,23 @@
       <c r="M28">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N28">
+        <v>0.21509</v>
+      </c>
+      <c r="O28">
+        <f>VLOOKUP(C28,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.426962734427077</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B29" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C29" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D29">
         <v>0</v>
@@ -3318,16 +3728,23 @@
       <c r="M29">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N29">
+        <v>2.5399999999999999E-2</v>
+      </c>
+      <c r="O29">
+        <f>VLOOKUP(C29,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.34718290865108348</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B30" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C30" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D30">
         <v>0</v>
@@ -3361,16 +3778,23 @@
       <c r="M30">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N30">
+        <v>0.35938000000000003</v>
+      </c>
+      <c r="O30">
+        <f>VLOOKUP(C30,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B31" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C31" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D31">
         <v>0</v>
@@ -3404,16 +3828,23 @@
       <c r="M31">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N31">
+        <v>0.33204999999999996</v>
+      </c>
+      <c r="O31">
+        <f>VLOOKUP(C31,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B32" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C32" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D32">
         <v>0</v>
@@ -3447,16 +3878,23 @@
       <c r="M32">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N32">
+        <v>0.44435999999999998</v>
+      </c>
+      <c r="O32">
+        <f>VLOOKUP(C32,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.28018755337085549</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B33" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C33" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D33">
         <v>0</v>
@@ -3490,16 +3928,23 @@
       <c r="M33">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N33">
+        <v>0.69155</v>
+      </c>
+      <c r="O33">
+        <f>VLOOKUP(C33,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.28018755337085549</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B34" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C34" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D34">
         <v>0</v>
@@ -3533,16 +3978,23 @@
       <c r="M34">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N34">
+        <v>0.35180999999999996</v>
+      </c>
+      <c r="O34">
+        <f>VLOOKUP(C34,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.42042078352794848</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B35" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C35" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D35">
         <v>0</v>
@@ -3576,16 +4028,23 @@
       <c r="M35">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N35">
+        <v>0.22187000000000001</v>
+      </c>
+      <c r="O35">
+        <f>VLOOKUP(C35,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B36" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C36" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D36">
         <v>0</v>
@@ -3619,16 +4078,23 @@
       <c r="M36">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N36">
+        <v>0.44503999999999999</v>
+      </c>
+      <c r="O36">
+        <f>VLOOKUP(C36,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B37" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C37" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D37">
         <v>0</v>
@@ -3662,16 +4128,23 @@
       <c r="M37">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N37">
+        <v>0.24213999999999999</v>
+      </c>
+      <c r="O37">
+        <f>VLOOKUP(C37,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B38" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C38" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D38">
         <v>0</v>
@@ -3705,16 +4178,23 @@
       <c r="M38">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N38">
+        <v>0.45749000000000001</v>
+      </c>
+      <c r="O38">
+        <f>VLOOKUP(C38,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B39" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C39" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D39">
         <v>0</v>
@@ -3748,16 +4228,23 @@
       <c r="M39">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N39">
+        <v>0.25361</v>
+      </c>
+      <c r="O39">
+        <f>VLOOKUP(C39,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.426962734427077</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B40" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C40" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D40">
         <v>0</v>
@@ -3791,16 +4278,23 @@
       <c r="M40">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N40">
+        <v>0.26077</v>
+      </c>
+      <c r="O40">
+        <f>VLOOKUP(C40,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.426962734427077</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B41" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C41" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D41">
         <v>0</v>
@@ -3834,16 +4328,23 @@
       <c r="M41">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N41">
+        <v>0.39161999999999997</v>
+      </c>
+      <c r="O41">
+        <f>VLOOKUP(C41,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.426962734427077</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B42" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C42" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D42">
         <v>0</v>
@@ -3877,16 +4378,23 @@
       <c r="M42">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N42">
+        <v>0.16811000000000001</v>
+      </c>
+      <c r="O42">
+        <f>VLOOKUP(C42,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.426962734427077</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B43" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C43" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D43">
         <v>0</v>
@@ -3920,16 +4428,23 @@
       <c r="M43">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N43">
+        <v>0.13964000000000001</v>
+      </c>
+      <c r="O43">
+        <f>VLOOKUP(C43,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.28018755337085549</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B44" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C44" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D44">
         <v>0</v>
@@ -3963,16 +4478,23 @@
       <c r="M44">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N44">
+        <v>0.15936</v>
+      </c>
+      <c r="O44">
+        <f>VLOOKUP(C44,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.35465693889566102</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B45" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C45" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D45">
         <v>0</v>
@@ -4006,16 +4528,23 @@
       <c r="M45">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N45">
+        <v>0.15195999999999998</v>
+      </c>
+      <c r="O45">
+        <f>VLOOKUP(C45,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.34718290865108348</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B46" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C46" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D46">
         <v>0</v>
@@ -4049,16 +4578,23 @@
       <c r="M46">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N46">
+        <v>0.12333</v>
+      </c>
+      <c r="O46">
+        <f>VLOOKUP(C46,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.34718290865108348</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B47" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C47" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D47">
         <v>0</v>
@@ -4092,16 +4628,23 @@
       <c r="M47">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N47">
+        <v>0.27202000000000004</v>
+      </c>
+      <c r="O47">
+        <f>VLOOKUP(C47,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.426962734427077</v>
+      </c>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B48" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C48" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D48">
         <v>0</v>
@@ -4135,16 +4678,23 @@
       <c r="M48">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N48">
+        <v>6.2619999999999995E-2</v>
+      </c>
+      <c r="O48">
+        <f>VLOOKUP(C48,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.34718290865108348</v>
+      </c>
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B49" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C49" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D49">
         <v>0</v>
@@ -4178,16 +4728,23 @@
       <c r="M49">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N49">
+        <v>0.22943999999999998</v>
+      </c>
+      <c r="O49">
+        <f>VLOOKUP(C49,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B50" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C50" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D50">
         <v>0</v>
@@ -4221,16 +4778,23 @@
       <c r="M50">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N50">
+        <v>0.23132000000000003</v>
+      </c>
+      <c r="O50">
+        <f>VLOOKUP(C50,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.42042078352794848</v>
+      </c>
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B51" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C51" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D51">
         <v>0</v>
@@ -4264,16 +4828,23 @@
       <c r="M51">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N51">
+        <v>0.30841000000000002</v>
+      </c>
+      <c r="O51">
+        <f>VLOOKUP(C51,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.28018755337085549</v>
+      </c>
+    </row>
+    <row r="52" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B52" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C52" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D52">
         <v>0</v>
@@ -4307,16 +4878,23 @@
       <c r="M52">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N52">
+        <v>0.33826999999999996</v>
+      </c>
+      <c r="O52">
+        <f>VLOOKUP(C52,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.28018755337085549</v>
+      </c>
+    </row>
+    <row r="53" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B53" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C53" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D53">
         <v>0</v>
@@ -4350,16 +4928,23 @@
       <c r="M53">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N53">
+        <v>0.67693999999999999</v>
+      </c>
+      <c r="O53">
+        <f>VLOOKUP(C53,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.28018755337085549</v>
+      </c>
+    </row>
+    <row r="54" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B54" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C54" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D54">
         <v>0</v>
@@ -4393,16 +4978,23 @@
       <c r="M54">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N54">
+        <v>0.40914</v>
+      </c>
+      <c r="O54">
+        <f>VLOOKUP(C54,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="55" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B55" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C55" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D55">
         <v>0</v>
@@ -4436,16 +5028,23 @@
       <c r="M55">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N55">
+        <v>0.14666999999999999</v>
+      </c>
+      <c r="O55">
+        <f>VLOOKUP(C55,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.35465693889566102</v>
+      </c>
+    </row>
+    <row r="56" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B56" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C56" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D56">
         <v>0</v>
@@ -4479,16 +5078,23 @@
       <c r="M56">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N56">
+        <v>0.59760000000000002</v>
+      </c>
+      <c r="O56">
+        <f>VLOOKUP(C56,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="57" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B57" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C57" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D57">
         <v>0</v>
@@ -4522,16 +5128,23 @@
       <c r="M57">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N57">
+        <v>0.21751000000000001</v>
+      </c>
+      <c r="O57">
+        <f>VLOOKUP(C57,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.34718290865108348</v>
+      </c>
+    </row>
+    <row r="58" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B58" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C58" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D58">
         <v>0</v>
@@ -4565,16 +5178,23 @@
       <c r="M58">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N58">
+        <v>0.46401999999999999</v>
+      </c>
+      <c r="O58">
+        <f>VLOOKUP(C58,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.42042078352794848</v>
+      </c>
+    </row>
+    <row r="59" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B59" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C59" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D59">
         <v>0</v>
@@ -4608,16 +5228,23 @@
       <c r="M59">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N59">
+        <v>0.55066999999999999</v>
+      </c>
+      <c r="O59">
+        <f>VLOOKUP(C59,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="60" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B60" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C60" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D60">
         <v>0</v>
@@ -4651,16 +5278,23 @@
       <c r="M60">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N60">
+        <v>0.48752000000000001</v>
+      </c>
+      <c r="O60">
+        <f>VLOOKUP(C60,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.28018755337085549</v>
+      </c>
+    </row>
+    <row r="61" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B61" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C61" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D61">
         <v>0</v>
@@ -4694,16 +5328,23 @@
       <c r="M61">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N61">
+        <v>0.28802</v>
+      </c>
+      <c r="O61">
+        <f>VLOOKUP(C61,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.42042078352794848</v>
+      </c>
+    </row>
+    <row r="62" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B62" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C62" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D62">
         <v>0</v>
@@ -4737,16 +5378,23 @@
       <c r="M62">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N62">
+        <v>0.50683999999999996</v>
+      </c>
+      <c r="O62">
+        <f>VLOOKUP(C62,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="63" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B63" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C63" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D63">
         <v>0</v>
@@ -4780,16 +5428,23 @@
       <c r="M63">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N63">
+        <v>0.30603999999999998</v>
+      </c>
+      <c r="O63">
+        <f>VLOOKUP(C63,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.35465693889566102</v>
+      </c>
+    </row>
+    <row r="64" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B64" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C64" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D64">
         <v>0</v>
@@ -4823,16 +5478,23 @@
       <c r="M64">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N64">
+        <v>0.28908</v>
+      </c>
+      <c r="O64">
+        <f>VLOOKUP(C64,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.28018755337085549</v>
+      </c>
+    </row>
+    <row r="65" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B65" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C65" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D65">
         <v>0</v>
@@ -4866,16 +5528,23 @@
       <c r="M65">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N65">
+        <v>0.4637</v>
+      </c>
+      <c r="O65">
+        <f>VLOOKUP(C65,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="66" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B66" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C66" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D66">
         <v>0</v>
@@ -4909,16 +5578,23 @@
       <c r="M66">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N66">
+        <v>0.39039000000000001</v>
+      </c>
+      <c r="O66">
+        <f>VLOOKUP(C66,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="67" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B67" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C67" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D67">
         <v>0</v>
@@ -4952,16 +5628,23 @@
       <c r="M67">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N67">
+        <v>0.29441000000000001</v>
+      </c>
+      <c r="O67">
+        <f>VLOOKUP(C67,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="68" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B68" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C68" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D68">
         <v>0</v>
@@ -4995,16 +5678,23 @@
       <c r="M68">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N68">
+        <v>0.56213000000000002</v>
+      </c>
+      <c r="O68">
+        <f>VLOOKUP(C68,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="69" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B69" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C69" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D69">
         <v>0</v>
@@ -5038,16 +5728,23 @@
       <c r="M69">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N69">
+        <v>0.4819</v>
+      </c>
+      <c r="O69">
+        <f>VLOOKUP(C69,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="70" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B70" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C70" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D70">
         <v>0</v>
@@ -5081,16 +5778,23 @@
       <c r="M70">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N70">
+        <v>0.18206</v>
+      </c>
+      <c r="O70">
+        <f>VLOOKUP(C70,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="71" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B71" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="C71" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D71">
         <v>0</v>
@@ -5124,16 +5828,23 @@
       <c r="M71">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N71">
+        <v>0.35310000000000002</v>
+      </c>
+      <c r="O71">
+        <f>VLOOKUP(C71,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.426962734427077</v>
+      </c>
+    </row>
+    <row r="72" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B72" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C72" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D72">
         <v>0</v>
@@ -5167,16 +5878,23 @@
       <c r="M72">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N72">
+        <v>0.26722000000000001</v>
+      </c>
+      <c r="O72">
+        <f>VLOOKUP(C72,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.35465693889566102</v>
+      </c>
+    </row>
+    <row r="73" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B73" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C73" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D73">
         <v>0</v>
@@ -5210,16 +5928,23 @@
       <c r="M73">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N73">
+        <v>0.10917</v>
+      </c>
+      <c r="O73">
+        <f>VLOOKUP(C73,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.34718290865108348</v>
+      </c>
+    </row>
+    <row r="74" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B74" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C74" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D74">
         <v>0</v>
@@ -5253,16 +5978,23 @@
       <c r="M74">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N74">
+        <v>0.2601</v>
+      </c>
+      <c r="O74">
+        <f>VLOOKUP(C74,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.426962734427077</v>
+      </c>
+    </row>
+    <row r="75" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B75" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C75" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D75">
         <v>0</v>
@@ -5296,16 +6028,23 @@
       <c r="M75">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N75">
+        <v>0.14777999999999999</v>
+      </c>
+      <c r="O75">
+        <f>VLOOKUP(C75,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.28018755337085549</v>
+      </c>
+    </row>
+    <row r="76" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B76" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C76" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D76">
         <v>0</v>
@@ -5339,16 +6078,23 @@
       <c r="M76">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N76">
+        <v>0.52139999999999997</v>
+      </c>
+      <c r="O76">
+        <f>VLOOKUP(C76,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.28018755337085549</v>
+      </c>
+    </row>
+    <row r="77" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B77" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C77" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D77">
         <v>0</v>
@@ -5382,16 +6128,23 @@
       <c r="M77">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N77">
+        <v>0.13516</v>
+      </c>
+      <c r="O77">
+        <f>VLOOKUP(C77,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.35465693889566102</v>
+      </c>
+    </row>
+    <row r="78" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B78" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C78" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D78">
         <v>0</v>
@@ -5425,16 +6178,23 @@
       <c r="M78">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N78">
+        <v>0.39335999999999999</v>
+      </c>
+      <c r="O78">
+        <f>VLOOKUP(C78,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.426962734427077</v>
+      </c>
+    </row>
+    <row r="79" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B79" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C79" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D79">
         <v>0</v>
@@ -5468,16 +6228,23 @@
       <c r="M79">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="80" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N79">
+        <v>5.9370000000000006E-2</v>
+      </c>
+      <c r="O79">
+        <f>VLOOKUP(C79,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="80" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B80" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C80" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D80">
         <v>0</v>
@@ -5511,16 +6278,23 @@
       <c r="M80">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N80">
+        <v>0.25389</v>
+      </c>
+      <c r="O80">
+        <f>VLOOKUP(C80,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.34718290865108348</v>
+      </c>
+    </row>
+    <row r="81" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B81" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C81" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D81">
         <v>0</v>
@@ -5554,16 +6328,23 @@
       <c r="M81">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="82" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N81">
+        <v>0.28386</v>
+      </c>
+      <c r="O81">
+        <f>VLOOKUP(C81,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="82" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B82" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C82" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D82">
         <v>0</v>
@@ -5597,16 +6378,23 @@
       <c r="M82">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="83" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N82">
+        <v>0.75946999999999998</v>
+      </c>
+      <c r="O82">
+        <f>VLOOKUP(C82,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.28018755337085549</v>
+      </c>
+    </row>
+    <row r="83" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B83" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C83" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D83">
         <v>0</v>
@@ -5640,16 +6428,23 @@
       <c r="M83">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="84" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N83">
+        <v>0.42259000000000002</v>
+      </c>
+      <c r="O83">
+        <f>VLOOKUP(C83,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="84" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B84" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C84" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D84">
         <v>0</v>
@@ -5683,16 +6478,23 @@
       <c r="M84">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="85" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N84">
+        <v>0.23346</v>
+      </c>
+      <c r="O84">
+        <f>VLOOKUP(C84,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.426962734427077</v>
+      </c>
+    </row>
+    <row r="85" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B85" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C85" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D85">
         <v>0</v>
@@ -5726,16 +6528,23 @@
       <c r="M85">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="86" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N85">
+        <v>0.17359000000000002</v>
+      </c>
+      <c r="O85">
+        <f>VLOOKUP(C85,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.34718290865108348</v>
+      </c>
+    </row>
+    <row r="86" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B86" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C86" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D86">
         <v>0</v>
@@ -5769,16 +6578,23 @@
       <c r="M86">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="87" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N86">
+        <v>0.34262999999999999</v>
+      </c>
+      <c r="O86">
+        <f>VLOOKUP(C86,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.42042078352794848</v>
+      </c>
+    </row>
+    <row r="87" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B87" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C87" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D87">
         <v>0</v>
@@ -5812,16 +6628,23 @@
       <c r="M87">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="88" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N87">
+        <v>0.34630000000000005</v>
+      </c>
+      <c r="O87">
+        <f>VLOOKUP(C87,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="88" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B88" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="C88" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D88">
         <v>0</v>
@@ -5855,16 +6678,23 @@
       <c r="M88">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="89" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N88">
+        <v>0.1583</v>
+      </c>
+      <c r="O88">
+        <f>VLOOKUP(C88,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="89" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B89" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="C89" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D89">
         <v>0</v>
@@ -5898,16 +6728,23 @@
       <c r="M89">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="90" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N89">
+        <v>0.75540999999999991</v>
+      </c>
+      <c r="O89">
+        <f>VLOOKUP(C89,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="90" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B90" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C90" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D90">
         <v>0</v>
@@ -5941,16 +6778,23 @@
       <c r="M90">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="91" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N90">
+        <v>0.18178</v>
+      </c>
+      <c r="O90">
+        <f>VLOOKUP(C90,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.34718290865108348</v>
+      </c>
+    </row>
+    <row r="91" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B91" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="C91" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D91">
         <v>0</v>
@@ -5984,16 +6828,23 @@
       <c r="M91">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="92" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N91">
+        <v>0.47659000000000001</v>
+      </c>
+      <c r="O91">
+        <f>VLOOKUP(C91,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="92" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B92" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C92" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D92">
         <v>0</v>
@@ -6027,16 +6878,23 @@
       <c r="M92">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="93" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N92">
+        <v>0.2661</v>
+      </c>
+      <c r="O92">
+        <f>VLOOKUP(C92,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="93" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B93" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="C93" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D93">
         <v>0</v>
@@ -6070,16 +6928,23 @@
       <c r="M93">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="94" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N93">
+        <v>0.37689</v>
+      </c>
+      <c r="O93">
+        <f>VLOOKUP(C93,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.35465693889566102</v>
+      </c>
+    </row>
+    <row r="94" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B94" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C94" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D94">
         <v>0</v>
@@ -6113,16 +6978,23 @@
       <c r="M94">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="95" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N94">
+        <v>0.15498000000000001</v>
+      </c>
+      <c r="O94">
+        <f>VLOOKUP(C94,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.42042078352794848</v>
+      </c>
+    </row>
+    <row r="95" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B95" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C95" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D95">
         <v>0</v>
@@ -6156,16 +7028,23 @@
       <c r="M95">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="96" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N95">
+        <v>0.21737999999999999</v>
+      </c>
+      <c r="O95">
+        <f>VLOOKUP(C95,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.42042078352794848</v>
+      </c>
+    </row>
+    <row r="96" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B96" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C96" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D96">
         <v>0</v>
@@ -6199,16 +7078,23 @@
       <c r="M96">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N96">
+        <v>0.48857</v>
+      </c>
+      <c r="O96">
+        <f>VLOOKUP(C96,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.35465693889566102</v>
+      </c>
+    </row>
+    <row r="97" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B97" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C97" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D97">
         <v>0</v>
@@ -6242,16 +7128,23 @@
       <c r="M97">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="98" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N97">
+        <v>0.39138000000000001</v>
+      </c>
+      <c r="O97">
+        <f>VLOOKUP(C97,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.28018755337085549</v>
+      </c>
+    </row>
+    <row r="98" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B98" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C98" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D98">
         <v>0</v>
@@ -6285,16 +7178,23 @@
       <c r="M98">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="99" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N98">
+        <v>0.28508</v>
+      </c>
+      <c r="O98">
+        <f>VLOOKUP(C98,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.34718290865108348</v>
+      </c>
+    </row>
+    <row r="99" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B99" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C99" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D99">
         <v>0</v>
@@ -6328,16 +7228,23 @@
       <c r="M99">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="100" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N99">
+        <v>0.25124999999999997</v>
+      </c>
+      <c r="O99">
+        <f>VLOOKUP(C99,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.28018755337085549</v>
+      </c>
+    </row>
+    <row r="100" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B100" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C100" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D100">
         <v>0</v>
@@ -6371,16 +7278,23 @@
       <c r="M100">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="101" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N100">
+        <v>0.41238999999999998</v>
+      </c>
+      <c r="O100">
+        <f>VLOOKUP(C100,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="101" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B101" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C101" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D101">
         <v>0</v>
@@ -6414,16 +7328,23 @@
       <c r="M101">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="102" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N101">
+        <v>0.23338</v>
+      </c>
+      <c r="O101">
+        <f>VLOOKUP(C101,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="102" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="B102" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C102" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D102">
         <v>0</v>
@@ -6457,16 +7378,23 @@
       <c r="M102">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="103" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N102">
+        <v>0.25289</v>
+      </c>
+      <c r="O102">
+        <f>VLOOKUP(C102,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.42042078352794848</v>
+      </c>
+    </row>
+    <row r="103" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B103" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C103" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D103">
         <v>0</v>
@@ -6500,16 +7428,23 @@
       <c r="M103">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="104" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N103">
+        <v>0.12848999999999999</v>
+      </c>
+      <c r="O103">
+        <f>VLOOKUP(C103,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.42042078352794848</v>
+      </c>
+    </row>
+    <row r="104" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="B104" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C104" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D104">
         <v>0</v>
@@ -6543,16 +7478,23 @@
       <c r="M104">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="105" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N104">
+        <v>0.11365</v>
+      </c>
+      <c r="O104">
+        <f>VLOOKUP(C104,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.426962734427077</v>
+      </c>
+    </row>
+    <row r="105" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B105" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C105" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D105">
         <v>0</v>
@@ -6586,16 +7528,23 @@
       <c r="M105">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="106" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N105">
+        <v>0.12478</v>
+      </c>
+      <c r="O105">
+        <f>VLOOKUP(C105,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.28018755337085549</v>
+      </c>
+    </row>
+    <row r="106" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B106" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C106" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D106">
         <v>0</v>
@@ -6629,16 +7578,23 @@
       <c r="M106">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="107" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N106">
+        <v>0.69864999999999999</v>
+      </c>
+      <c r="O106">
+        <f>VLOOKUP(C106,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.28018755337085549</v>
+      </c>
+    </row>
+    <row r="107" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B107" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C107" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D107">
         <v>0</v>
@@ -6672,16 +7628,23 @@
       <c r="M107">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="108" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N107">
+        <v>0.41828000000000004</v>
+      </c>
+      <c r="O107">
+        <f>VLOOKUP(C107,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.28018755337085549</v>
+      </c>
+    </row>
+    <row r="108" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B108" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C108" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D108">
         <v>0</v>
@@ -6715,16 +7678,23 @@
       <c r="M108">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="109" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N108">
+        <v>0.15273</v>
+      </c>
+      <c r="O108">
+        <f>VLOOKUP(C108,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.34718290865108348</v>
+      </c>
+    </row>
+    <row r="109" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="B109" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C109" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D109">
         <v>0</v>
@@ -6758,16 +7728,23 @@
       <c r="M109">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="110" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N109">
+        <v>0.20541000000000001</v>
+      </c>
+      <c r="O109">
+        <f>VLOOKUP(C109,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="110" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B110" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C110" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D110">
         <v>0</v>
@@ -6801,16 +7778,23 @@
       <c r="M110">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="111" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N110">
+        <v>0.44965000000000005</v>
+      </c>
+      <c r="O110">
+        <f>VLOOKUP(C110,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
+      </c>
+    </row>
+    <row r="111" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="B111" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C111" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D111">
         <v>0</v>
@@ -6843,6 +7827,13 @@
       </c>
       <c r="M111">
         <v>0.5</v>
+      </c>
+      <c r="N111">
+        <v>0.65342</v>
+      </c>
+      <c r="O111">
+        <f>VLOOKUP(C111,WHO_region_parameters!$A$2:$D$7,4,FALSE)*Dx_infacilitytesting_acceptability</f>
+        <v>0.26594516366578902</v>
       </c>
     </row>
   </sheetData>
@@ -6852,199 +7843,416 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DA8E731-11F0-484A-B543-F518ABE10A2B}">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="34.7265625" customWidth="1"/>
-    <col min="3" max="3" width="80.26953125" customWidth="1"/>
+    <col min="3" max="3" width="48.36328125" customWidth="1"/>
+    <col min="4" max="4" width="80.26953125" customWidth="1"/>
+    <col min="5" max="5" width="28" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="E1" s="1" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A2" s="6" t="s">
         <v>305</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="6" t="s">
-        <v>307</v>
       </c>
       <c r="B2">
         <v>0.92</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+        <v>369</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="E2" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="B3">
         <v>0.6</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="32.15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>370</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="32.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="B4">
         <v>0.9</v>
       </c>
-      <c r="C4" s="9" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C4" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="B5">
         <v>2026</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+        <v>374</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="B6">
         <v>2029</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+        <v>375</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="B7">
         <v>0.9</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+        <v>376</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="B8">
         <v>0.9</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="6" t="s">
+        <v>315</v>
+      </c>
+      <c r="B9">
+        <v>0.5</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>316</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" s="6" t="s">
-        <v>319</v>
-      </c>
-      <c r="B9">
-        <v>0.5</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="B10">
         <v>2028</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C10" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="B11">
         <v>2031</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="B12">
+        <v>2028</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="D12" s="5"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="B13">
+        <v>2032</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" s="6" t="s">
+        <v>319</v>
+      </c>
+      <c r="B14">
+        <v>0.6</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>320</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="6" t="s">
-        <v>357</v>
-      </c>
-      <c r="B12">
-        <v>2027</v>
-      </c>
-      <c r="C12" s="5"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" s="6" t="s">
-        <v>358</v>
-      </c>
-      <c r="B13">
-        <v>2028</v>
-      </c>
-      <c r="C13" s="5"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" s="6" t="s">
-        <v>323</v>
-      </c>
-      <c r="B14">
-        <v>0.6</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="B15">
         <v>30</v>
       </c>
-      <c r="C15" s="5" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D15" s="5" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="B16">
-        <v>99</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+        <v>100</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="6" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="B17">
         <v>5</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>330</v>
+      <c r="D17" s="2" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A18" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="B18">
+        <v>0.5</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A19" s="6" t="s">
+        <v>403</v>
+      </c>
+      <c r="B19">
+        <v>0</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A20" s="6" t="s">
+        <v>404</v>
+      </c>
+      <c r="B20">
+        <v>0.8</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A21" s="6" t="s">
+        <v>401</v>
+      </c>
+      <c r="B21">
+        <v>0.05</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A22" s="6" t="s">
+        <v>402</v>
+      </c>
+      <c r="B22">
+        <v>0.8</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A23" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="B23">
+        <v>0</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" s="6" t="s">
+        <v>386</v>
+      </c>
+      <c r="B24">
+        <v>0.01</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A25" s="6" t="s">
+        <v>391</v>
+      </c>
+      <c r="B25">
+        <v>0.5</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A26" s="6" t="s">
+        <v>392</v>
+      </c>
+      <c r="B26">
+        <v>0.5</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A27" s="6" t="s">
+        <v>396</v>
+      </c>
+      <c r="B27">
+        <v>0</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A28" s="6" t="s">
+        <v>393</v>
+      </c>
+      <c r="B28">
+        <v>0.01</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A29" s="6" t="s">
+        <v>394</v>
+      </c>
+      <c r="B29">
+        <v>0.5</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A30" s="6" t="s">
+        <v>395</v>
+      </c>
+      <c r="B30">
+        <v>0.5</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" s="6" t="s">
+        <v>410</v>
+      </c>
+      <c r="B31">
+        <v>0.6</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A32" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="B32">
+        <v>0.2</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>413</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C4" r:id="rId1" xr:uid="{6C608058-9D31-4C99-ADB5-8E8AF527D663}"/>
+    <hyperlink ref="D4" r:id="rId1" xr:uid="{6C608058-9D31-4C99-ADB5-8E8AF527D663}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId2"/>
@@ -7053,83 +8261,102 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{503939F2-1EAC-4666-A91D-ABC857B0018A}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.453125" customWidth="1"/>
     <col min="2" max="2" width="26.81640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="30" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+        <v>328</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B2">
         <v>4.0000000000000001E-3</v>
       </c>
       <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0.53189032733157804</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B3">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="C3">
+        <v>3.0999999999999999E-3</v>
+      </c>
+      <c r="D3">
+        <v>0.85392546885415399</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B4">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="C4">
         <v>1.2500000000000001E-2</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>84</v>
-      </c>
-      <c r="B3">
-        <v>4.0000000000000001E-3</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>87</v>
-      </c>
-      <c r="B4">
+      <c r="D4">
+        <v>0.69436581730216695</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B5">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="C4">
+      <c r="C5">
         <v>1.2699999999999999E-2</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>100</v>
-      </c>
-      <c r="B5">
+      <c r="D5">
+        <v>0.84084156705589697</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>98</v>
+      </c>
+      <c r="B6">
         <v>0.01</v>
       </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>107</v>
-      </c>
-      <c r="B6">
-        <v>7.0000000000000001E-3</v>
-      </c>
       <c r="C6">
-        <v>3.0999999999999999E-3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0.70931387779132204</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B7">
         <v>1.6E-2</v>
@@ -7137,6 +8364,51 @@
       <c r="C7">
         <v>3.8E-3</v>
       </c>
+      <c r="D7">
+        <v>0.56037510674171098</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E11" s="14"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E12" s="14"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E13" s="15"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E14" s="15"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E15" s="15"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E16" s="15"/>
+    </row>
+    <row r="17" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E17" s="15"/>
+    </row>
+    <row r="18" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E18" s="15"/>
+    </row>
+    <row r="19" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E19" s="15"/>
+    </row>
+    <row r="20" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E20" s="15"/>
+    </row>
+    <row r="21" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E21" s="15"/>
+    </row>
+    <row r="22" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E22" s="15"/>
+    </row>
+    <row r="23" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E23" s="15"/>
+    </row>
+    <row r="24" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E24" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7145,12 +8417,32 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A53FDAB6-3CC6-4A73-81DA-060E35532B9E}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>333</v>
+        <v>329</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>360</v>
       </c>
     </row>
   </sheetData>

</xml_diff>